<commit_message>
Updated investors data file
</commit_message>
<xml_diff>
--- a/investors.xlsx
+++ b/investors.xlsx
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1370,63 +1373,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nikhil</t>
+          <t>Harshala Patole</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1212121212</v>
+        <v>987457352</v>
       </c>
       <c r="C2" s="1" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>jmd 6.0</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="D2" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>jmd 6.0</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="H2" s="1" t="n">
-        <v>46166</v>
-      </c>
-      <c r="I2" t="b">
-        <v>1</v>
-      </c>
-      <c r="J2" s="1" t="n">
-        <v>46163</v>
-      </c>
       <c r="K2" t="b">
         <v>0</v>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" s="1" t="n">
+        <v>46174</v>
+      </c>
       <c r="N2" t="b">
         <v>0</v>
       </c>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" s="1" t="n">
+        <v>46204</v>
+      </c>
       <c r="Q2" t="b">
         <v>0</v>
       </c>
       <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
+      <c r="S2" s="1" t="n">
+        <v>46235</v>
+      </c>
       <c r="T2" t="b">
         <v>0</v>
       </c>
       <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+      <c r="V2" s="1" t="n">
+        <v>46266</v>
+      </c>
       <c r="W2" t="b">
         <v>0</v>
       </c>
       <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
+      <c r="Y2" s="1" t="n">
+        <v>46296</v>
+      </c>
       <c r="Z2" t="b">
         <v>0</v>
       </c>
@@ -1705,332 +1718,264 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Satish Patole</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" s="1" t="n">
+          <t>Ajay Bhosale</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>9874623097</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>jmd 6.0</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" s="2" t="n">
         <v>46143</v>
       </c>
-      <c r="D3" t="n">
-        <v>200000</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G3" t="n">
-        <v>100000</v>
-      </c>
-      <c r="H3" s="1" t="n">
-        <v>46265</v>
-      </c>
-      <c r="I3" t="b">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>46165</v>
-      </c>
-      <c r="K3" t="b">
-        <v>0</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" s="1" t="n">
-        <v>46192</v>
-      </c>
       <c r="N3" t="b">
         <v>0</v>
       </c>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="P3" s="2" t="n">
+        <v>46174</v>
+      </c>
       <c r="Q3" t="b">
         <v>0</v>
       </c>
       <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+      <c r="S3" s="2" t="n">
+        <v>46204</v>
+      </c>
       <c r="T3" t="b">
         <v>0</v>
       </c>
       <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
+      <c r="V3" s="2" t="n">
+        <v>46235</v>
+      </c>
       <c r="W3" t="b">
         <v>0</v>
       </c>
       <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
+      <c r="Y3" s="2" t="n">
+        <v>46235</v>
+      </c>
       <c r="Z3" t="b">
         <v>0</v>
       </c>
       <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
+      <c r="AB3" s="2" t="n">
+        <v>46266</v>
+      </c>
       <c r="AC3" t="b">
         <v>0</v>
       </c>
       <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AE3" s="2" t="n">
+        <v>46296</v>
+      </c>
       <c r="AF3" t="b">
         <v>0</v>
       </c>
       <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
+      <c r="AH3" s="2" t="n">
+        <v>46327</v>
+      </c>
       <c r="AI3" t="b">
         <v>0</v>
       </c>
       <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
+      <c r="AK3" s="2" t="n">
+        <v>46357</v>
+      </c>
       <c r="AL3" t="b">
         <v>0</v>
       </c>
       <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
+      <c r="AN3" s="2" t="n">
+        <v>46388</v>
+      </c>
       <c r="AO3" t="b">
         <v>0</v>
       </c>
       <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
+      <c r="AQ3" s="2" t="n">
+        <v>46419</v>
+      </c>
       <c r="AR3" t="b">
         <v>0</v>
       </c>
       <c r="AS3" t="inlineStr"/>
       <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="b">
-        <v>0</v>
-      </c>
+      <c r="AU3" t="inlineStr"/>
       <c r="AV3" t="inlineStr"/>
       <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="b">
-        <v>0</v>
-      </c>
+      <c r="AX3" t="inlineStr"/>
       <c r="AY3" t="inlineStr"/>
       <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="b">
-        <v>0</v>
-      </c>
+      <c r="BA3" t="inlineStr"/>
       <c r="BB3" t="inlineStr"/>
       <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="b">
-        <v>0</v>
-      </c>
+      <c r="BD3" t="inlineStr"/>
       <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="inlineStr"/>
-      <c r="BG3" t="b">
-        <v>0</v>
-      </c>
+      <c r="BG3" t="inlineStr"/>
       <c r="BH3" t="inlineStr"/>
       <c r="BI3" t="inlineStr"/>
-      <c r="BJ3" t="b">
-        <v>0</v>
-      </c>
+      <c r="BJ3" t="inlineStr"/>
       <c r="BK3" t="inlineStr"/>
       <c r="BL3" t="inlineStr"/>
-      <c r="BM3" t="b">
-        <v>0</v>
-      </c>
+      <c r="BM3" t="inlineStr"/>
       <c r="BN3" t="inlineStr"/>
       <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="b">
-        <v>0</v>
-      </c>
+      <c r="BP3" t="inlineStr"/>
       <c r="BQ3" t="inlineStr"/>
       <c r="BR3" t="inlineStr"/>
-      <c r="BS3" t="b">
-        <v>0</v>
-      </c>
+      <c r="BS3" t="inlineStr"/>
       <c r="BT3" t="inlineStr"/>
       <c r="BU3" t="inlineStr"/>
-      <c r="BV3" t="b">
-        <v>0</v>
-      </c>
+      <c r="BV3" t="inlineStr"/>
       <c r="BW3" t="inlineStr"/>
       <c r="BX3" t="inlineStr"/>
-      <c r="BY3" t="b">
-        <v>0</v>
-      </c>
+      <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
       <c r="CA3" t="inlineStr"/>
-      <c r="CB3" t="b">
-        <v>0</v>
-      </c>
+      <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr"/>
       <c r="CD3" t="inlineStr"/>
-      <c r="CE3" t="b">
-        <v>0</v>
-      </c>
+      <c r="CE3" t="inlineStr"/>
       <c r="CF3" t="inlineStr"/>
       <c r="CG3" t="inlineStr"/>
-      <c r="CH3" t="b">
-        <v>0</v>
-      </c>
+      <c r="CH3" t="inlineStr"/>
       <c r="CI3" t="inlineStr"/>
       <c r="CJ3" t="inlineStr"/>
-      <c r="CK3" t="b">
-        <v>0</v>
-      </c>
+      <c r="CK3" t="inlineStr"/>
       <c r="CL3" t="inlineStr"/>
       <c r="CM3" t="inlineStr"/>
-      <c r="CN3" t="b">
-        <v>0</v>
-      </c>
+      <c r="CN3" t="inlineStr"/>
       <c r="CO3" t="inlineStr"/>
       <c r="CP3" t="inlineStr"/>
-      <c r="CQ3" t="b">
-        <v>0</v>
-      </c>
+      <c r="CQ3" t="inlineStr"/>
       <c r="CR3" t="inlineStr"/>
       <c r="CS3" t="inlineStr"/>
-      <c r="CT3" t="b">
-        <v>0</v>
-      </c>
+      <c r="CT3" t="inlineStr"/>
       <c r="CU3" t="inlineStr"/>
       <c r="CV3" t="inlineStr"/>
-      <c r="CW3" t="b">
-        <v>0</v>
-      </c>
+      <c r="CW3" t="inlineStr"/>
       <c r="CX3" t="inlineStr"/>
       <c r="CY3" t="inlineStr"/>
-      <c r="CZ3" t="b">
-        <v>0</v>
-      </c>
+      <c r="CZ3" t="inlineStr"/>
       <c r="DA3" t="inlineStr"/>
       <c r="DB3" t="inlineStr"/>
-      <c r="DC3" t="b">
-        <v>0</v>
-      </c>
+      <c r="DC3" t="inlineStr"/>
       <c r="DD3" t="inlineStr"/>
       <c r="DE3" t="inlineStr"/>
-      <c r="DF3" t="b">
-        <v>0</v>
-      </c>
+      <c r="DF3" t="inlineStr"/>
       <c r="DG3" t="inlineStr"/>
       <c r="DH3" t="inlineStr"/>
-      <c r="DI3" t="b">
-        <v>0</v>
-      </c>
+      <c r="DI3" t="inlineStr"/>
       <c r="DJ3" t="inlineStr"/>
       <c r="DK3" t="inlineStr"/>
-      <c r="DL3" t="b">
-        <v>0</v>
-      </c>
+      <c r="DL3" t="inlineStr"/>
       <c r="DM3" t="inlineStr"/>
       <c r="DN3" t="inlineStr"/>
-      <c r="DO3" t="b">
-        <v>0</v>
-      </c>
+      <c r="DO3" t="inlineStr"/>
       <c r="DP3" t="inlineStr"/>
       <c r="DQ3" t="inlineStr"/>
-      <c r="DR3" t="b">
-        <v>0</v>
-      </c>
+      <c r="DR3" t="inlineStr"/>
       <c r="DS3" t="inlineStr"/>
       <c r="DT3" t="inlineStr"/>
-      <c r="DU3" t="b">
-        <v>0</v>
-      </c>
+      <c r="DU3" t="inlineStr"/>
       <c r="DV3" t="inlineStr"/>
       <c r="DW3" t="inlineStr"/>
-      <c r="DX3" t="b">
-        <v>0</v>
-      </c>
+      <c r="DX3" t="inlineStr"/>
       <c r="DY3" t="inlineStr"/>
       <c r="DZ3" t="inlineStr"/>
-      <c r="EA3" t="b">
-        <v>0</v>
-      </c>
+      <c r="EA3" t="inlineStr"/>
       <c r="EB3" t="inlineStr"/>
       <c r="EC3" t="inlineStr"/>
-      <c r="ED3" t="b">
-        <v>0</v>
-      </c>
+      <c r="ED3" t="inlineStr"/>
       <c r="EE3" t="inlineStr"/>
       <c r="EF3" t="inlineStr"/>
-      <c r="EG3" t="b">
-        <v>0</v>
-      </c>
+      <c r="EG3" t="inlineStr"/>
       <c r="EH3" t="inlineStr"/>
       <c r="EI3" t="inlineStr"/>
-      <c r="EJ3" t="b">
-        <v>0</v>
-      </c>
+      <c r="EJ3" t="inlineStr"/>
       <c r="EK3" t="inlineStr"/>
       <c r="EL3" t="inlineStr"/>
-      <c r="EM3" t="b">
-        <v>0</v>
-      </c>
+      <c r="EM3" t="inlineStr"/>
       <c r="EN3" t="inlineStr"/>
       <c r="EO3" t="inlineStr"/>
-      <c r="EP3" t="b">
-        <v>0</v>
-      </c>
+      <c r="EP3" t="inlineStr"/>
       <c r="EQ3" t="inlineStr"/>
       <c r="ER3" t="inlineStr"/>
-      <c r="ES3" t="b">
-        <v>0</v>
-      </c>
+      <c r="ES3" t="inlineStr"/>
       <c r="ET3" t="inlineStr"/>
       <c r="EU3" t="inlineStr"/>
-      <c r="EV3" t="b">
-        <v>0</v>
-      </c>
+      <c r="EV3" t="inlineStr"/>
       <c r="EW3" t="inlineStr"/>
       <c r="EX3" t="inlineStr"/>
-      <c r="EY3" t="b">
-        <v>0</v>
-      </c>
+      <c r="EY3" t="inlineStr"/>
       <c r="EZ3" t="inlineStr"/>
       <c r="FA3" t="inlineStr"/>
-      <c r="FB3" t="b">
-        <v>0</v>
-      </c>
+      <c r="FB3" t="inlineStr"/>
       <c r="FC3" t="inlineStr"/>
       <c r="FD3" t="inlineStr"/>
-      <c r="FE3" t="b">
-        <v>0</v>
-      </c>
+      <c r="FE3" t="inlineStr"/>
       <c r="FF3" t="inlineStr"/>
       <c r="FG3" t="inlineStr"/>
-      <c r="FH3" t="b">
-        <v>0</v>
-      </c>
+      <c r="FH3" t="inlineStr"/>
       <c r="FI3" t="inlineStr"/>
       <c r="FJ3" t="inlineStr"/>
-      <c r="FK3" t="b">
-        <v>0</v>
-      </c>
+      <c r="FK3" t="inlineStr"/>
       <c r="FL3" t="inlineStr"/>
       <c r="FM3" t="inlineStr"/>
-      <c r="FN3" t="b">
-        <v>0</v>
-      </c>
+      <c r="FN3" t="inlineStr"/>
       <c r="FO3" t="inlineStr"/>
       <c r="FP3" t="inlineStr"/>
-      <c r="FQ3" t="b">
-        <v>0</v>
-      </c>
+      <c r="FQ3" t="inlineStr"/>
       <c r="FR3" t="inlineStr"/>
       <c r="FS3" t="inlineStr"/>
-      <c r="FT3" t="b">
-        <v>0</v>
-      </c>
+      <c r="FT3" t="inlineStr"/>
       <c r="FU3" t="inlineStr"/>
       <c r="FV3" t="inlineStr"/>
-      <c r="FW3" t="b">
-        <v>0</v>
-      </c>
+      <c r="FW3" t="inlineStr"/>
       <c r="FX3" t="inlineStr"/>
       <c r="FY3" t="inlineStr"/>
-      <c r="FZ3" t="b">
-        <v>0</v>
-      </c>
+      <c r="FZ3" t="inlineStr"/>
       <c r="GA3" t="inlineStr"/>
       <c r="GB3" t="inlineStr"/>
-      <c r="GC3" t="b">
-        <v>0</v>
-      </c>
+      <c r="GC3" t="inlineStr"/>
       <c r="GD3" t="inlineStr"/>
       <c r="GE3" t="inlineStr"/>
-      <c r="GF3" t="b">
-        <v>0</v>
-      </c>
+      <c r="GF3" t="inlineStr"/>
       <c r="GG3" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>